<commit_message>
feat(excel): add step scaling experiments (4k..1024k) marked as unrun
</commit_message>
<xml_diff>
--- a/ALL_DOCS_EXPERIMENTS_CONFIG_TO_RESULTS.xlsx
+++ b/ALL_DOCS_EXPERIMENTS_CONFIG_TO_RESULTS.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -65,8 +65,14 @@
       <color rgb="00D0D0D0"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00B25900"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -128,6 +134,11 @@
         <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -169,7 +180,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -245,6 +256,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -611,11 +625,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW127"/>
+  <dimension ref="A1:AW133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
@@ -675,7 +689,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>共 124 项实验统一按序号 001..124 顺序排列</t>
+          <t>共 130 项实验统一按序号 001..130 顺序排列</t>
         </is>
       </c>
     </row>
@@ -29567,6 +29581,1392 @@
       <c r="AW127" s="25" t="inlineStr">
         <is>
           <t>GRPO组内相对优势极其稳定，4位加法提升5pp且减法无回退。</t>
+        </is>
+      </c>
+    </row>
+    <row r="128" ht="24" customHeight="1">
+      <c r="A128" s="9" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+      <c r="B128" s="10" t="inlineStr">
+        <is>
+          <t>【步数扩展-长周期训练】L4_D128 CoT 4,000步基线 (待运行)</t>
+        </is>
+      </c>
+      <c r="C128" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="D128" s="11" t="n">
+        <v>128</v>
+      </c>
+      <c r="E128" s="11" t="n">
+        <v>4000</v>
+      </c>
+      <c r="F128" s="11" t="n">
+        <v>32</v>
+      </c>
+      <c r="G128" s="11" t="n">
+        <v>4000</v>
+      </c>
+      <c r="H128" s="11" t="inlineStr">
+        <is>
+          <t>128.0</t>
+        </is>
+      </c>
+      <c r="I128" s="11" t="n">
+        <v>128000</v>
+      </c>
+      <c r="J128" s="10" t="inlineStr">
+        <is>
+          <t>动态生成器 (加减竖式)</t>
+        </is>
+      </c>
+      <c r="K128" s="12" t="inlineStr">
+        <is>
+          <t>1-4位</t>
+        </is>
+      </c>
+      <c r="L128" s="12" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="M128" s="12" t="inlineStr">
+        <is>
+          <t>无衰减</t>
+        </is>
+      </c>
+      <c r="N128" s="12" t="inlineStr">
+        <is>
+          <t>0..3 随机</t>
+        </is>
+      </c>
+      <c r="O128" s="11" t="inlineStr">
+        <is>
+          <t>3e-4</t>
+        </is>
+      </c>
+      <c r="P128" s="10" t="inlineStr">
+        <is>
+          <t>Cosine + Warmup</t>
+        </is>
+      </c>
+      <c r="Q128" s="11" t="n">
+        <v>200</v>
+      </c>
+      <c r="R128" s="11" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="S128" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T128" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U128" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="V128" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="W128" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="X128" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y128" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z128" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AA128" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AB128" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AC128" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AD128" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE128" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AF128" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AG128" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AH128" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AI128" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AJ128" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AK128" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AL128" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AM128" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AN128" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AO128" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AP128" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AQ128" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AR128" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AS128" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AT128" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AU128" s="18" t="inlineStr">
+        <is>
+          <t>固定测试集 (n=40)</t>
+        </is>
+      </c>
+      <c r="AV128" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AW128" s="19" t="inlineStr">
+        <is>
+          <t>【待运行 / 未跑】计划验证 4,000 步基线收敛表现。</t>
+        </is>
+      </c>
+    </row>
+    <row r="129" ht="24" customHeight="1">
+      <c r="A129" s="20" t="inlineStr">
+        <is>
+          <t>126</t>
+        </is>
+      </c>
+      <c r="B129" s="21" t="inlineStr">
+        <is>
+          <t>【步数扩展-长周期训练】L4_D128 CoT 8,000步扩展 (待运行)</t>
+        </is>
+      </c>
+      <c r="C129" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="D129" s="22" t="n">
+        <v>128</v>
+      </c>
+      <c r="E129" s="22" t="n">
+        <v>8000</v>
+      </c>
+      <c r="F129" s="22" t="n">
+        <v>32</v>
+      </c>
+      <c r="G129" s="22" t="n">
+        <v>8000</v>
+      </c>
+      <c r="H129" s="22" t="inlineStr">
+        <is>
+          <t>256.0</t>
+        </is>
+      </c>
+      <c r="I129" s="22" t="n">
+        <v>256000</v>
+      </c>
+      <c r="J129" s="21" t="inlineStr">
+        <is>
+          <t>动态生成器 (加减竖式)</t>
+        </is>
+      </c>
+      <c r="K129" s="23" t="inlineStr">
+        <is>
+          <t>1-4位</t>
+        </is>
+      </c>
+      <c r="L129" s="23" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="M129" s="23" t="inlineStr">
+        <is>
+          <t>无衰减</t>
+        </is>
+      </c>
+      <c r="N129" s="23" t="inlineStr">
+        <is>
+          <t>0..3 随机</t>
+        </is>
+      </c>
+      <c r="O129" s="22" t="inlineStr">
+        <is>
+          <t>3e-4</t>
+        </is>
+      </c>
+      <c r="P129" s="21" t="inlineStr">
+        <is>
+          <t>Cosine + Warmup</t>
+        </is>
+      </c>
+      <c r="Q129" s="22" t="n">
+        <v>200</v>
+      </c>
+      <c r="R129" s="22" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="S129" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T129" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U129" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="V129" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="W129" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="X129" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y129" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z129" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AA129" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AB129" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AC129" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AD129" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE129" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AF129" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AG129" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AH129" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AI129" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AJ129" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AK129" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AL129" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AM129" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AN129" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AO129" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AP129" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AQ129" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AR129" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AS129" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AT129" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AU129" s="16" t="inlineStr">
+        <is>
+          <t>固定测试集 (n=40)</t>
+        </is>
+      </c>
+      <c r="AV129" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AW129" s="25" t="inlineStr">
+        <is>
+          <t>【待运行 / 未跑】计划验证 8,000 步翻倍训练对4位减法与难例进位的增益。</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" ht="24" customHeight="1">
+      <c r="A130" s="9" t="inlineStr">
+        <is>
+          <t>127</t>
+        </is>
+      </c>
+      <c r="B130" s="10" t="inlineStr">
+        <is>
+          <t>【步数扩展-长周期训练】L4_D128 CoT 16,000步扩展 (待运行)</t>
+        </is>
+      </c>
+      <c r="C130" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="D130" s="11" t="n">
+        <v>128</v>
+      </c>
+      <c r="E130" s="11" t="n">
+        <v>16000</v>
+      </c>
+      <c r="F130" s="11" t="n">
+        <v>32</v>
+      </c>
+      <c r="G130" s="11" t="n">
+        <v>16000</v>
+      </c>
+      <c r="H130" s="11" t="inlineStr">
+        <is>
+          <t>512.0</t>
+        </is>
+      </c>
+      <c r="I130" s="11" t="n">
+        <v>512000</v>
+      </c>
+      <c r="J130" s="10" t="inlineStr">
+        <is>
+          <t>动态生成器 (加减竖式)</t>
+        </is>
+      </c>
+      <c r="K130" s="12" t="inlineStr">
+        <is>
+          <t>1-4位</t>
+        </is>
+      </c>
+      <c r="L130" s="12" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="M130" s="12" t="inlineStr">
+        <is>
+          <t>无衰减</t>
+        </is>
+      </c>
+      <c r="N130" s="12" t="inlineStr">
+        <is>
+          <t>0..3 随机</t>
+        </is>
+      </c>
+      <c r="O130" s="11" t="inlineStr">
+        <is>
+          <t>3e-4</t>
+        </is>
+      </c>
+      <c r="P130" s="10" t="inlineStr">
+        <is>
+          <t>Cosine + Warmup</t>
+        </is>
+      </c>
+      <c r="Q130" s="11" t="n">
+        <v>200</v>
+      </c>
+      <c r="R130" s="11" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="S130" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T130" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U130" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="V130" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="W130" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="X130" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y130" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z130" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AA130" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AB130" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AC130" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AD130" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE130" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AF130" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AG130" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AH130" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AI130" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AJ130" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AK130" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AL130" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AM130" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AN130" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AO130" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AP130" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AQ130" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AR130" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AS130" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AT130" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AU130" s="18" t="inlineStr">
+        <is>
+          <t>固定测试集 (n=40)</t>
+        </is>
+      </c>
+      <c r="AV130" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AW130" s="19" t="inlineStr">
+        <is>
+          <t>【待运行 / 未跑】计划验证 16,000 步长程训练下的损失下限与稳定性。</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" ht="24" customHeight="1">
+      <c r="A131" s="20" t="inlineStr">
+        <is>
+          <t>128</t>
+        </is>
+      </c>
+      <c r="B131" s="21" t="inlineStr">
+        <is>
+          <t>【步数扩展-长周期训练】L4_D128 CoT 32,000步扩展 (待运行)</t>
+        </is>
+      </c>
+      <c r="C131" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="D131" s="22" t="n">
+        <v>128</v>
+      </c>
+      <c r="E131" s="22" t="n">
+        <v>32000</v>
+      </c>
+      <c r="F131" s="22" t="n">
+        <v>32</v>
+      </c>
+      <c r="G131" s="22" t="n">
+        <v>32000</v>
+      </c>
+      <c r="H131" s="22" t="inlineStr">
+        <is>
+          <t>1024.0</t>
+        </is>
+      </c>
+      <c r="I131" s="22" t="n">
+        <v>1024000</v>
+      </c>
+      <c r="J131" s="21" t="inlineStr">
+        <is>
+          <t>动态生成器 (加减竖式)</t>
+        </is>
+      </c>
+      <c r="K131" s="23" t="inlineStr">
+        <is>
+          <t>1-4位</t>
+        </is>
+      </c>
+      <c r="L131" s="23" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="M131" s="23" t="inlineStr">
+        <is>
+          <t>无衰减</t>
+        </is>
+      </c>
+      <c r="N131" s="23" t="inlineStr">
+        <is>
+          <t>0..3 随机</t>
+        </is>
+      </c>
+      <c r="O131" s="22" t="inlineStr">
+        <is>
+          <t>3e-4</t>
+        </is>
+      </c>
+      <c r="P131" s="21" t="inlineStr">
+        <is>
+          <t>Cosine + Warmup</t>
+        </is>
+      </c>
+      <c r="Q131" s="22" t="n">
+        <v>200</v>
+      </c>
+      <c r="R131" s="22" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="S131" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T131" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U131" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="V131" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="W131" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="X131" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y131" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z131" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AA131" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AB131" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AC131" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AD131" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE131" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AF131" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AG131" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AH131" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AI131" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AJ131" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AK131" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AL131" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AM131" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AN131" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AO131" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AP131" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AQ131" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AR131" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AS131" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AT131" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AU131" s="16" t="inlineStr">
+        <is>
+          <t>固定测试集 (n=40)</t>
+        </is>
+      </c>
+      <c r="AV131" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AW131" s="25" t="inlineStr">
+        <is>
+          <t>【待运行 / 未跑】计划验证 32,000 步下是否存在过拟合或退化现象。</t>
+        </is>
+      </c>
+    </row>
+    <row r="132" ht="24" customHeight="1">
+      <c r="A132" s="9" t="inlineStr">
+        <is>
+          <t>129</t>
+        </is>
+      </c>
+      <c r="B132" s="10" t="inlineStr">
+        <is>
+          <t>【步数扩展-长周期训练】L4_D128 CoT 128,000步超长训练 (待运行)</t>
+        </is>
+      </c>
+      <c r="C132" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="D132" s="11" t="n">
+        <v>128</v>
+      </c>
+      <c r="E132" s="11" t="n">
+        <v>128000</v>
+      </c>
+      <c r="F132" s="11" t="n">
+        <v>32</v>
+      </c>
+      <c r="G132" s="11" t="n">
+        <v>128000</v>
+      </c>
+      <c r="H132" s="11" t="inlineStr">
+        <is>
+          <t>4096.0</t>
+        </is>
+      </c>
+      <c r="I132" s="11" t="n">
+        <v>4096000</v>
+      </c>
+      <c r="J132" s="10" t="inlineStr">
+        <is>
+          <t>动态生成器 (加减竖式)</t>
+        </is>
+      </c>
+      <c r="K132" s="12" t="inlineStr">
+        <is>
+          <t>1-4位</t>
+        </is>
+      </c>
+      <c r="L132" s="12" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="M132" s="12" t="inlineStr">
+        <is>
+          <t>无衰减</t>
+        </is>
+      </c>
+      <c r="N132" s="12" t="inlineStr">
+        <is>
+          <t>0..3 随机</t>
+        </is>
+      </c>
+      <c r="O132" s="11" t="inlineStr">
+        <is>
+          <t>3e-4</t>
+        </is>
+      </c>
+      <c r="P132" s="10" t="inlineStr">
+        <is>
+          <t>Cosine + Warmup</t>
+        </is>
+      </c>
+      <c r="Q132" s="11" t="n">
+        <v>200</v>
+      </c>
+      <c r="R132" s="11" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="S132" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T132" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U132" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="V132" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="W132" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="X132" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y132" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z132" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AA132" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AB132" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AC132" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AD132" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE132" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AF132" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AG132" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AH132" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AI132" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AJ132" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AK132" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AL132" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AM132" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AN132" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AO132" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AP132" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AQ132" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AR132" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AS132" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AT132" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AU132" s="18" t="inlineStr">
+        <is>
+          <t>固定测试集 (n=40)</t>
+        </is>
+      </c>
+      <c r="AV132" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AW132" s="19" t="inlineStr">
+        <is>
+          <t>【待运行 / 未跑】计划验证 128,000 步超长训练的缩放定律（Scaling Law）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="133" ht="24" customHeight="1">
+      <c r="A133" s="20" t="inlineStr">
+        <is>
+          <t>130</t>
+        </is>
+      </c>
+      <c r="B133" s="21" t="inlineStr">
+        <is>
+          <t>【步数扩展-长周期训练】L4_D128 CoT 1,024,000步极限吞吐测试 (待运行)</t>
+        </is>
+      </c>
+      <c r="C133" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="D133" s="22" t="n">
+        <v>128</v>
+      </c>
+      <c r="E133" s="22" t="n">
+        <v>1024000</v>
+      </c>
+      <c r="F133" s="22" t="n">
+        <v>32</v>
+      </c>
+      <c r="G133" s="22" t="n">
+        <v>1024000</v>
+      </c>
+      <c r="H133" s="22" t="inlineStr">
+        <is>
+          <t>32768.0</t>
+        </is>
+      </c>
+      <c r="I133" s="22" t="n">
+        <v>32768000</v>
+      </c>
+      <c r="J133" s="21" t="inlineStr">
+        <is>
+          <t>动态生成器 (加减竖式)</t>
+        </is>
+      </c>
+      <c r="K133" s="23" t="inlineStr">
+        <is>
+          <t>1-4位</t>
+        </is>
+      </c>
+      <c r="L133" s="23" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="M133" s="23" t="inlineStr">
+        <is>
+          <t>无衰减</t>
+        </is>
+      </c>
+      <c r="N133" s="23" t="inlineStr">
+        <is>
+          <t>0..3 随机</t>
+        </is>
+      </c>
+      <c r="O133" s="22" t="inlineStr">
+        <is>
+          <t>3e-4</t>
+        </is>
+      </c>
+      <c r="P133" s="21" t="inlineStr">
+        <is>
+          <t>Cosine + Warmup</t>
+        </is>
+      </c>
+      <c r="Q133" s="22" t="n">
+        <v>200</v>
+      </c>
+      <c r="R133" s="22" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="S133" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T133" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U133" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="V133" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="W133" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="X133" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y133" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z133" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AA133" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AB133" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AC133" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AD133" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE133" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AF133" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AG133" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AH133" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AI133" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AJ133" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AK133" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AL133" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AM133" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AN133" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AO133" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AP133" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AQ133" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AR133" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AS133" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AT133" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AU133" s="16" t="inlineStr">
+        <is>
+          <t>固定测试集 (n=40)</t>
+        </is>
+      </c>
+      <c r="AV133" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AW133" s="25" t="inlineStr">
+        <is>
+          <t>【待运行 / 未跑】计划验证 1,024,000 步（1M+ 步）极限算力下的泛化上限。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(excel): add comprehensive step gradient experiments (20..1024k) marked as unrun
</commit_message>
<xml_diff>
--- a/ALL_DOCS_EXPERIMENTS_CONFIG_TO_RESULTS.xlsx
+++ b/ALL_DOCS_EXPERIMENTS_CONFIG_TO_RESULTS.xlsx
@@ -625,7 +625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW133"/>
+  <dimension ref="A1:AW143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -689,7 +689,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>共 130 项实验统一按序号 001..130 顺序排列</t>
+          <t>共 140 项实验统一按序号 001..140 顺序排列</t>
         </is>
       </c>
     </row>
@@ -23648,7 +23648,7 @@
         </is>
       </c>
       <c r="Q102" s="11" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="R102" s="11" t="n">
         <v>0.1</v>
@@ -24572,7 +24572,7 @@
         </is>
       </c>
       <c r="Q106" s="11" t="n">
-        <v>200</v>
+        <v>162</v>
       </c>
       <c r="R106" s="11" t="n">
         <v>0.1</v>
@@ -25496,7 +25496,7 @@
         </is>
       </c>
       <c r="Q110" s="11" t="n">
-        <v>200</v>
+        <v>162</v>
       </c>
       <c r="R110" s="11" t="n">
         <v>0.1</v>
@@ -27344,7 +27344,7 @@
         </is>
       </c>
       <c r="Q118" s="11" t="n">
-        <v>200</v>
+        <v>37</v>
       </c>
       <c r="R118" s="11" t="n">
         <v>0.1</v>
@@ -27575,7 +27575,7 @@
         </is>
       </c>
       <c r="Q119" s="22" t="n">
-        <v>200</v>
+        <v>37</v>
       </c>
       <c r="R119" s="22" t="n">
         <v>0.1</v>
@@ -27806,7 +27806,7 @@
         </is>
       </c>
       <c r="Q120" s="11" t="n">
-        <v>200</v>
+        <v>37</v>
       </c>
       <c r="R120" s="11" t="n">
         <v>0.1</v>
@@ -28037,7 +28037,7 @@
         </is>
       </c>
       <c r="Q121" s="22" t="n">
-        <v>200</v>
+        <v>37</v>
       </c>
       <c r="R121" s="22" t="n">
         <v>0.1</v>
@@ -28268,7 +28268,7 @@
         </is>
       </c>
       <c r="Q122" s="11" t="n">
-        <v>200</v>
+        <v>37</v>
       </c>
       <c r="R122" s="11" t="n">
         <v>0.1</v>
@@ -28499,7 +28499,7 @@
         </is>
       </c>
       <c r="Q123" s="22" t="n">
-        <v>200</v>
+        <v>37</v>
       </c>
       <c r="R123" s="22" t="n">
         <v>0.1</v>
@@ -28730,7 +28730,7 @@
         </is>
       </c>
       <c r="Q124" s="11" t="n">
-        <v>200</v>
+        <v>75</v>
       </c>
       <c r="R124" s="11" t="n">
         <v>0.1</v>
@@ -28961,7 +28961,7 @@
         </is>
       </c>
       <c r="Q125" s="22" t="n">
-        <v>200</v>
+        <v>37</v>
       </c>
       <c r="R125" s="22" t="n">
         <v>0.1</v>
@@ -29192,7 +29192,7 @@
         </is>
       </c>
       <c r="Q126" s="11" t="n">
-        <v>200</v>
+        <v>37</v>
       </c>
       <c r="R126" s="11" t="n">
         <v>0.1</v>
@@ -29423,7 +29423,7 @@
         </is>
       </c>
       <c r="Q127" s="22" t="n">
-        <v>200</v>
+        <v>37</v>
       </c>
       <c r="R127" s="22" t="n">
         <v>0.1</v>
@@ -29592,7 +29592,7 @@
       </c>
       <c r="B128" s="10" t="inlineStr">
         <is>
-          <t>【步数扩展-长周期训练】L4_D128 CoT 4,000步基线 (待运行)</t>
+          <t>【步数扩展-梯度扫描】L4_D128 CoT 20步 极速收敛探针 (待运行)</t>
         </is>
       </c>
       <c r="C128" s="11" t="n">
@@ -29602,21 +29602,21 @@
         <v>128</v>
       </c>
       <c r="E128" s="11" t="n">
-        <v>4000</v>
+        <v>20</v>
       </c>
       <c r="F128" s="11" t="n">
         <v>32</v>
       </c>
       <c r="G128" s="11" t="n">
-        <v>4000</v>
+        <v>20</v>
       </c>
       <c r="H128" s="11" t="inlineStr">
         <is>
-          <t>128.0</t>
+          <t>0.6</t>
         </is>
       </c>
       <c r="I128" s="11" t="n">
-        <v>128000</v>
+        <v>640</v>
       </c>
       <c r="J128" s="10" t="inlineStr">
         <is>
@@ -29654,7 +29654,7 @@
         </is>
       </c>
       <c r="Q128" s="11" t="n">
-        <v>200</v>
+        <v>5</v>
       </c>
       <c r="R128" s="11" t="n">
         <v>0.1</v>
@@ -29811,7 +29811,7 @@
       </c>
       <c r="AW128" s="19" t="inlineStr">
         <is>
-          <t>【待运行 / 未跑】计划验证 4,000 步基线收敛表现。</t>
+          <t>【待运行 / 未跑】计划在 Colab 上评估 20 步训练的损失收敛与多位算术准确率。</t>
         </is>
       </c>
     </row>
@@ -29823,7 +29823,7 @@
       </c>
       <c r="B129" s="21" t="inlineStr">
         <is>
-          <t>【步数扩展-长周期训练】L4_D128 CoT 8,000步扩展 (待运行)</t>
+          <t>【步数扩展-梯度扫描】L4_D128 CoT 50步 冒烟基线探针 (待运行)</t>
         </is>
       </c>
       <c r="C129" s="22" t="n">
@@ -29833,21 +29833,21 @@
         <v>128</v>
       </c>
       <c r="E129" s="22" t="n">
-        <v>8000</v>
+        <v>50</v>
       </c>
       <c r="F129" s="22" t="n">
         <v>32</v>
       </c>
       <c r="G129" s="22" t="n">
-        <v>8000</v>
+        <v>50</v>
       </c>
       <c r="H129" s="22" t="inlineStr">
         <is>
-          <t>256.0</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="I129" s="22" t="n">
-        <v>256000</v>
+        <v>1600</v>
       </c>
       <c r="J129" s="21" t="inlineStr">
         <is>
@@ -29885,7 +29885,7 @@
         </is>
       </c>
       <c r="Q129" s="22" t="n">
-        <v>200</v>
+        <v>12</v>
       </c>
       <c r="R129" s="22" t="n">
         <v>0.1</v>
@@ -30042,7 +30042,7 @@
       </c>
       <c r="AW129" s="25" t="inlineStr">
         <is>
-          <t>【待运行 / 未跑】计划验证 8,000 步翻倍训练对4位减法与难例进位的增益。</t>
+          <t>【待运行 / 未跑】计划在 Colab 上评估 50 步训练的损失收敛与多位算术准确率。</t>
         </is>
       </c>
     </row>
@@ -30054,7 +30054,7 @@
       </c>
       <c r="B130" s="10" t="inlineStr">
         <is>
-          <t>【步数扩展-长周期训练】L4_D128 CoT 16,000步扩展 (待运行)</t>
+          <t>【步数扩展-梯度扫描】L4_D128 CoT 100步 初期对齐探针 (待运行)</t>
         </is>
       </c>
       <c r="C130" s="11" t="n">
@@ -30064,21 +30064,21 @@
         <v>128</v>
       </c>
       <c r="E130" s="11" t="n">
-        <v>16000</v>
+        <v>100</v>
       </c>
       <c r="F130" s="11" t="n">
         <v>32</v>
       </c>
       <c r="G130" s="11" t="n">
-        <v>16000</v>
+        <v>100</v>
       </c>
       <c r="H130" s="11" t="inlineStr">
         <is>
-          <t>512.0</t>
+          <t>3.2</t>
         </is>
       </c>
       <c r="I130" s="11" t="n">
-        <v>512000</v>
+        <v>3200</v>
       </c>
       <c r="J130" s="10" t="inlineStr">
         <is>
@@ -30116,7 +30116,7 @@
         </is>
       </c>
       <c r="Q130" s="11" t="n">
-        <v>200</v>
+        <v>25</v>
       </c>
       <c r="R130" s="11" t="n">
         <v>0.1</v>
@@ -30273,7 +30273,7 @@
       </c>
       <c r="AW130" s="19" t="inlineStr">
         <is>
-          <t>【待运行 / 未跑】计划验证 16,000 步长程训练下的损失下限与稳定性。</t>
+          <t>【待运行 / 未跑】计划在 Colab 上评估 100 步训练的损失收敛与多位算术准确率。</t>
         </is>
       </c>
     </row>
@@ -30285,7 +30285,7 @@
       </c>
       <c r="B131" s="21" t="inlineStr">
         <is>
-          <t>【步数扩展-长周期训练】L4_D128 CoT 32,000步扩展 (待运行)</t>
+          <t>【步数扩展-梯度扫描】L4_D128 CoT 200步 早期学习探针 (待运行)</t>
         </is>
       </c>
       <c r="C131" s="22" t="n">
@@ -30295,21 +30295,21 @@
         <v>128</v>
       </c>
       <c r="E131" s="22" t="n">
-        <v>32000</v>
+        <v>200</v>
       </c>
       <c r="F131" s="22" t="n">
         <v>32</v>
       </c>
       <c r="G131" s="22" t="n">
-        <v>32000</v>
+        <v>200</v>
       </c>
       <c r="H131" s="22" t="inlineStr">
         <is>
-          <t>1024.0</t>
+          <t>6.4</t>
         </is>
       </c>
       <c r="I131" s="22" t="n">
-        <v>1024000</v>
+        <v>6400</v>
       </c>
       <c r="J131" s="21" t="inlineStr">
         <is>
@@ -30347,7 +30347,7 @@
         </is>
       </c>
       <c r="Q131" s="22" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="R131" s="22" t="n">
         <v>0.1</v>
@@ -30504,7 +30504,7 @@
       </c>
       <c r="AW131" s="25" t="inlineStr">
         <is>
-          <t>【待运行 / 未跑】计划验证 32,000 步下是否存在过拟合或退化现象。</t>
+          <t>【待运行 / 未跑】计划在 Colab 上评估 200 步训练的损失收敛与多位算术准确率。</t>
         </is>
       </c>
     </row>
@@ -30516,7 +30516,7 @@
       </c>
       <c r="B132" s="10" t="inlineStr">
         <is>
-          <t>【步数扩展-长周期训练】L4_D128 CoT 128,000步超长训练 (待运行)</t>
+          <t>【步数扩展-梯度扫描】L4_D128 CoT 500步 初步收敛探针 (待运行)</t>
         </is>
       </c>
       <c r="C132" s="11" t="n">
@@ -30526,21 +30526,21 @@
         <v>128</v>
       </c>
       <c r="E132" s="11" t="n">
-        <v>128000</v>
+        <v>500</v>
       </c>
       <c r="F132" s="11" t="n">
         <v>32</v>
       </c>
       <c r="G132" s="11" t="n">
-        <v>128000</v>
+        <v>500</v>
       </c>
       <c r="H132" s="11" t="inlineStr">
         <is>
-          <t>4096.0</t>
+          <t>16.0</t>
         </is>
       </c>
       <c r="I132" s="11" t="n">
-        <v>4096000</v>
+        <v>16000</v>
       </c>
       <c r="J132" s="10" t="inlineStr">
         <is>
@@ -30578,7 +30578,7 @@
         </is>
       </c>
       <c r="Q132" s="11" t="n">
-        <v>200</v>
+        <v>125</v>
       </c>
       <c r="R132" s="11" t="n">
         <v>0.1</v>
@@ -30735,7 +30735,7 @@
       </c>
       <c r="AW132" s="19" t="inlineStr">
         <is>
-          <t>【待运行 / 未跑】计划验证 128,000 步超长训练的缩放定律（Scaling Law）。</t>
+          <t>【待运行 / 未跑】计划在 Colab 上评估 500 步训练的损失收敛与多位算术准确率。</t>
         </is>
       </c>
     </row>
@@ -30747,7 +30747,7 @@
       </c>
       <c r="B133" s="21" t="inlineStr">
         <is>
-          <t>【步数扩展-长周期训练】L4_D128 CoT 1,024,000步极限吞吐测试 (待运行)</t>
+          <t>【步数扩展-梯度扫描】L4_D128 CoT 1,000步 早期阶段基线 (待运行)</t>
         </is>
       </c>
       <c r="C133" s="22" t="n">
@@ -30757,21 +30757,21 @@
         <v>128</v>
       </c>
       <c r="E133" s="22" t="n">
-        <v>1024000</v>
+        <v>1000</v>
       </c>
       <c r="F133" s="22" t="n">
         <v>32</v>
       </c>
       <c r="G133" s="22" t="n">
-        <v>1024000</v>
+        <v>1000</v>
       </c>
       <c r="H133" s="22" t="inlineStr">
         <is>
-          <t>32768.0</t>
+          <t>32.0</t>
         </is>
       </c>
       <c r="I133" s="22" t="n">
-        <v>32768000</v>
+        <v>32000</v>
       </c>
       <c r="J133" s="21" t="inlineStr">
         <is>
@@ -30966,7 +30966,2317 @@
       </c>
       <c r="AW133" s="25" t="inlineStr">
         <is>
-          <t>【待运行 / 未跑】计划验证 1,024,000 步（1M+ 步）极限算力下的泛化上限。</t>
+          <t>【待运行 / 未跑】计划在 Colab 上评估 1,000 步训练的损失收敛与多位算术准确率。</t>
+        </is>
+      </c>
+    </row>
+    <row r="134" ht="24" customHeight="1">
+      <c r="A134" s="9" t="inlineStr">
+        <is>
+          <t>131</t>
+        </is>
+      </c>
+      <c r="B134" s="10" t="inlineStr">
+        <is>
+          <t>【步数扩展-梯度扫描】L4_D128 CoT 2,000步 半程收敛探针 (待运行)</t>
+        </is>
+      </c>
+      <c r="C134" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="D134" s="11" t="n">
+        <v>128</v>
+      </c>
+      <c r="E134" s="11" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F134" s="11" t="n">
+        <v>32</v>
+      </c>
+      <c r="G134" s="11" t="n">
+        <v>2000</v>
+      </c>
+      <c r="H134" s="11" t="inlineStr">
+        <is>
+          <t>64.0</t>
+        </is>
+      </c>
+      <c r="I134" s="11" t="n">
+        <v>64000</v>
+      </c>
+      <c r="J134" s="10" t="inlineStr">
+        <is>
+          <t>动态生成器 (加减竖式)</t>
+        </is>
+      </c>
+      <c r="K134" s="12" t="inlineStr">
+        <is>
+          <t>1-4位</t>
+        </is>
+      </c>
+      <c r="L134" s="12" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="M134" s="12" t="inlineStr">
+        <is>
+          <t>无衰减</t>
+        </is>
+      </c>
+      <c r="N134" s="12" t="inlineStr">
+        <is>
+          <t>0..3 随机</t>
+        </is>
+      </c>
+      <c r="O134" s="11" t="inlineStr">
+        <is>
+          <t>3e-4</t>
+        </is>
+      </c>
+      <c r="P134" s="10" t="inlineStr">
+        <is>
+          <t>Cosine + Warmup</t>
+        </is>
+      </c>
+      <c r="Q134" s="11" t="n">
+        <v>200</v>
+      </c>
+      <c r="R134" s="11" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="S134" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T134" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U134" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="V134" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="W134" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="X134" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y134" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z134" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AA134" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AB134" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AC134" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AD134" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE134" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AF134" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AG134" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AH134" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AI134" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AJ134" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AK134" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AL134" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AM134" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AN134" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AO134" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AP134" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AQ134" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AR134" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AS134" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AT134" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AU134" s="18" t="inlineStr">
+        <is>
+          <t>固定测试集 (n=40)</t>
+        </is>
+      </c>
+      <c r="AV134" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AW134" s="19" t="inlineStr">
+        <is>
+          <t>【待运行 / 未跑】计划在 Colab 上评估 2,000 步训练的损失收敛与多位算术准确率。</t>
+        </is>
+      </c>
+    </row>
+    <row r="135" ht="24" customHeight="1">
+      <c r="A135" s="20" t="inlineStr">
+        <is>
+          <t>132</t>
+        </is>
+      </c>
+      <c r="B135" s="21" t="inlineStr">
+        <is>
+          <t>【步数扩展-梯度扫描】L4_D128 CoT 4,000步 标准基线 (待运行)</t>
+        </is>
+      </c>
+      <c r="C135" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="D135" s="22" t="n">
+        <v>128</v>
+      </c>
+      <c r="E135" s="22" t="n">
+        <v>4000</v>
+      </c>
+      <c r="F135" s="22" t="n">
+        <v>32</v>
+      </c>
+      <c r="G135" s="22" t="n">
+        <v>4000</v>
+      </c>
+      <c r="H135" s="22" t="inlineStr">
+        <is>
+          <t>128.0</t>
+        </is>
+      </c>
+      <c r="I135" s="22" t="n">
+        <v>128000</v>
+      </c>
+      <c r="J135" s="21" t="inlineStr">
+        <is>
+          <t>动态生成器 (加减竖式)</t>
+        </is>
+      </c>
+      <c r="K135" s="23" t="inlineStr">
+        <is>
+          <t>1-4位</t>
+        </is>
+      </c>
+      <c r="L135" s="23" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="M135" s="23" t="inlineStr">
+        <is>
+          <t>无衰减</t>
+        </is>
+      </c>
+      <c r="N135" s="23" t="inlineStr">
+        <is>
+          <t>0..3 随机</t>
+        </is>
+      </c>
+      <c r="O135" s="22" t="inlineStr">
+        <is>
+          <t>3e-4</t>
+        </is>
+      </c>
+      <c r="P135" s="21" t="inlineStr">
+        <is>
+          <t>Cosine + Warmup</t>
+        </is>
+      </c>
+      <c r="Q135" s="22" t="n">
+        <v>200</v>
+      </c>
+      <c r="R135" s="22" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="S135" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T135" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U135" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="V135" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="W135" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="X135" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y135" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z135" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AA135" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AB135" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AC135" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AD135" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE135" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AF135" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AG135" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AH135" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AI135" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AJ135" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AK135" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AL135" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AM135" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AN135" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AO135" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AP135" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AQ135" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AR135" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AS135" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AT135" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AU135" s="16" t="inlineStr">
+        <is>
+          <t>固定测试集 (n=40)</t>
+        </is>
+      </c>
+      <c r="AV135" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AW135" s="25" t="inlineStr">
+        <is>
+          <t>【待运行 / 未跑】计划在 Colab 上评估 4,000 步训练的损失收敛与多位算术准确率。</t>
+        </is>
+      </c>
+    </row>
+    <row r="136" ht="24" customHeight="1">
+      <c r="A136" s="9" t="inlineStr">
+        <is>
+          <t>133</t>
+        </is>
+      </c>
+      <c r="B136" s="10" t="inlineStr">
+        <is>
+          <t>【步数扩展-梯度扫描】L4_D128 CoT 8,000步 翻倍扩展 (待运行)</t>
+        </is>
+      </c>
+      <c r="C136" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="D136" s="11" t="n">
+        <v>128</v>
+      </c>
+      <c r="E136" s="11" t="n">
+        <v>8000</v>
+      </c>
+      <c r="F136" s="11" t="n">
+        <v>32</v>
+      </c>
+      <c r="G136" s="11" t="n">
+        <v>8000</v>
+      </c>
+      <c r="H136" s="11" t="inlineStr">
+        <is>
+          <t>256.0</t>
+        </is>
+      </c>
+      <c r="I136" s="11" t="n">
+        <v>256000</v>
+      </c>
+      <c r="J136" s="10" t="inlineStr">
+        <is>
+          <t>动态生成器 (加减竖式)</t>
+        </is>
+      </c>
+      <c r="K136" s="12" t="inlineStr">
+        <is>
+          <t>1-4位</t>
+        </is>
+      </c>
+      <c r="L136" s="12" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="M136" s="12" t="inlineStr">
+        <is>
+          <t>无衰减</t>
+        </is>
+      </c>
+      <c r="N136" s="12" t="inlineStr">
+        <is>
+          <t>0..3 随机</t>
+        </is>
+      </c>
+      <c r="O136" s="11" t="inlineStr">
+        <is>
+          <t>3e-4</t>
+        </is>
+      </c>
+      <c r="P136" s="10" t="inlineStr">
+        <is>
+          <t>Cosine + Warmup</t>
+        </is>
+      </c>
+      <c r="Q136" s="11" t="n">
+        <v>200</v>
+      </c>
+      <c r="R136" s="11" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="S136" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T136" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U136" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="V136" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="W136" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="X136" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y136" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z136" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AA136" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AB136" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AC136" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AD136" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE136" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AF136" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AG136" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AH136" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AI136" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AJ136" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AK136" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AL136" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AM136" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AN136" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AO136" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AP136" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AQ136" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AR136" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AS136" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AT136" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AU136" s="18" t="inlineStr">
+        <is>
+          <t>固定测试集 (n=40)</t>
+        </is>
+      </c>
+      <c r="AV136" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AW136" s="19" t="inlineStr">
+        <is>
+          <t>【待运行 / 未跑】计划在 Colab 上评估 8,000 步训练的损失收敛与多位算术准确率。</t>
+        </is>
+      </c>
+    </row>
+    <row r="137" ht="24" customHeight="1">
+      <c r="A137" s="20" t="inlineStr">
+        <is>
+          <t>134</t>
+        </is>
+      </c>
+      <c r="B137" s="21" t="inlineStr">
+        <is>
+          <t>【步数扩展-梯度扫描】L4_D128 CoT 16,000步 长程扩展 (待运行)</t>
+        </is>
+      </c>
+      <c r="C137" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="D137" s="22" t="n">
+        <v>128</v>
+      </c>
+      <c r="E137" s="22" t="n">
+        <v>16000</v>
+      </c>
+      <c r="F137" s="22" t="n">
+        <v>32</v>
+      </c>
+      <c r="G137" s="22" t="n">
+        <v>16000</v>
+      </c>
+      <c r="H137" s="22" t="inlineStr">
+        <is>
+          <t>512.0</t>
+        </is>
+      </c>
+      <c r="I137" s="22" t="n">
+        <v>512000</v>
+      </c>
+      <c r="J137" s="21" t="inlineStr">
+        <is>
+          <t>动态生成器 (加减竖式)</t>
+        </is>
+      </c>
+      <c r="K137" s="23" t="inlineStr">
+        <is>
+          <t>1-4位</t>
+        </is>
+      </c>
+      <c r="L137" s="23" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="M137" s="23" t="inlineStr">
+        <is>
+          <t>无衰减</t>
+        </is>
+      </c>
+      <c r="N137" s="23" t="inlineStr">
+        <is>
+          <t>0..3 随机</t>
+        </is>
+      </c>
+      <c r="O137" s="22" t="inlineStr">
+        <is>
+          <t>3e-4</t>
+        </is>
+      </c>
+      <c r="P137" s="21" t="inlineStr">
+        <is>
+          <t>Cosine + Warmup</t>
+        </is>
+      </c>
+      <c r="Q137" s="22" t="n">
+        <v>200</v>
+      </c>
+      <c r="R137" s="22" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="S137" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T137" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U137" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="V137" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="W137" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="X137" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y137" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z137" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AA137" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AB137" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AC137" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AD137" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE137" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AF137" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AG137" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AH137" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AI137" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AJ137" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AK137" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AL137" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AM137" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AN137" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AO137" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AP137" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AQ137" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AR137" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AS137" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AT137" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AU137" s="16" t="inlineStr">
+        <is>
+          <t>固定测试集 (n=40)</t>
+        </is>
+      </c>
+      <c r="AV137" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AW137" s="25" t="inlineStr">
+        <is>
+          <t>【待运行 / 未跑】计划在 Colab 上评估 16,000 步训练的损失收敛与多位算术准确率。</t>
+        </is>
+      </c>
+    </row>
+    <row r="138" ht="24" customHeight="1">
+      <c r="A138" s="9" t="inlineStr">
+        <is>
+          <t>135</t>
+        </is>
+      </c>
+      <c r="B138" s="10" t="inlineStr">
+        <is>
+          <t>【步数扩展-梯度扫描】L4_D128 CoT 32,000步 深度训练 (待运行)</t>
+        </is>
+      </c>
+      <c r="C138" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="D138" s="11" t="n">
+        <v>128</v>
+      </c>
+      <c r="E138" s="11" t="n">
+        <v>32000</v>
+      </c>
+      <c r="F138" s="11" t="n">
+        <v>32</v>
+      </c>
+      <c r="G138" s="11" t="n">
+        <v>32000</v>
+      </c>
+      <c r="H138" s="11" t="inlineStr">
+        <is>
+          <t>1024.0</t>
+        </is>
+      </c>
+      <c r="I138" s="11" t="n">
+        <v>1024000</v>
+      </c>
+      <c r="J138" s="10" t="inlineStr">
+        <is>
+          <t>动态生成器 (加减竖式)</t>
+        </is>
+      </c>
+      <c r="K138" s="12" t="inlineStr">
+        <is>
+          <t>1-4位</t>
+        </is>
+      </c>
+      <c r="L138" s="12" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="M138" s="12" t="inlineStr">
+        <is>
+          <t>无衰减</t>
+        </is>
+      </c>
+      <c r="N138" s="12" t="inlineStr">
+        <is>
+          <t>0..3 随机</t>
+        </is>
+      </c>
+      <c r="O138" s="11" t="inlineStr">
+        <is>
+          <t>3e-4</t>
+        </is>
+      </c>
+      <c r="P138" s="10" t="inlineStr">
+        <is>
+          <t>Cosine + Warmup</t>
+        </is>
+      </c>
+      <c r="Q138" s="11" t="n">
+        <v>200</v>
+      </c>
+      <c r="R138" s="11" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="S138" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T138" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U138" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="V138" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="W138" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="X138" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y138" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z138" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AA138" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AB138" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AC138" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AD138" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE138" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AF138" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AG138" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AH138" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AI138" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AJ138" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AK138" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AL138" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AM138" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AN138" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AO138" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AP138" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AQ138" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AR138" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AS138" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AT138" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AU138" s="18" t="inlineStr">
+        <is>
+          <t>固定测试集 (n=40)</t>
+        </is>
+      </c>
+      <c r="AV138" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AW138" s="19" t="inlineStr">
+        <is>
+          <t>【待运行 / 未跑】计划在 Colab 上评估 32,000 步训练的损失收敛与多位算术准确率。</t>
+        </is>
+      </c>
+    </row>
+    <row r="139" ht="24" customHeight="1">
+      <c r="A139" s="20" t="inlineStr">
+        <is>
+          <t>136</t>
+        </is>
+      </c>
+      <c r="B139" s="21" t="inlineStr">
+        <is>
+          <t>【步数扩展-梯度扫描】L4_D128 CoT 64,000步 超长训练 (待运行)</t>
+        </is>
+      </c>
+      <c r="C139" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="D139" s="22" t="n">
+        <v>128</v>
+      </c>
+      <c r="E139" s="22" t="n">
+        <v>64000</v>
+      </c>
+      <c r="F139" s="22" t="n">
+        <v>32</v>
+      </c>
+      <c r="G139" s="22" t="n">
+        <v>64000</v>
+      </c>
+      <c r="H139" s="22" t="inlineStr">
+        <is>
+          <t>2048.0</t>
+        </is>
+      </c>
+      <c r="I139" s="22" t="n">
+        <v>2048000</v>
+      </c>
+      <c r="J139" s="21" t="inlineStr">
+        <is>
+          <t>动态生成器 (加减竖式)</t>
+        </is>
+      </c>
+      <c r="K139" s="23" t="inlineStr">
+        <is>
+          <t>1-4位</t>
+        </is>
+      </c>
+      <c r="L139" s="23" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="M139" s="23" t="inlineStr">
+        <is>
+          <t>无衰减</t>
+        </is>
+      </c>
+      <c r="N139" s="23" t="inlineStr">
+        <is>
+          <t>0..3 随机</t>
+        </is>
+      </c>
+      <c r="O139" s="22" t="inlineStr">
+        <is>
+          <t>3e-4</t>
+        </is>
+      </c>
+      <c r="P139" s="21" t="inlineStr">
+        <is>
+          <t>Cosine + Warmup</t>
+        </is>
+      </c>
+      <c r="Q139" s="22" t="n">
+        <v>200</v>
+      </c>
+      <c r="R139" s="22" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="S139" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T139" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U139" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="V139" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="W139" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="X139" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y139" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z139" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AA139" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AB139" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AC139" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AD139" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE139" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AF139" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AG139" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AH139" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AI139" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AJ139" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AK139" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AL139" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AM139" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AN139" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AO139" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AP139" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AQ139" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AR139" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AS139" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AT139" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AU139" s="16" t="inlineStr">
+        <is>
+          <t>固定测试集 (n=40)</t>
+        </is>
+      </c>
+      <c r="AV139" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AW139" s="25" t="inlineStr">
+        <is>
+          <t>【待运行 / 未跑】计划在 Colab 上评估 64,000 步训练的损失收敛与多位算术准确率。</t>
+        </is>
+      </c>
+    </row>
+    <row r="140" ht="24" customHeight="1">
+      <c r="A140" s="9" t="inlineStr">
+        <is>
+          <t>137</t>
+        </is>
+      </c>
+      <c r="B140" s="10" t="inlineStr">
+        <is>
+          <t>【步数扩展-梯度扫描】L4_D128 CoT 128,000步 缩放扫描 (待运行)</t>
+        </is>
+      </c>
+      <c r="C140" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="D140" s="11" t="n">
+        <v>128</v>
+      </c>
+      <c r="E140" s="11" t="n">
+        <v>128000</v>
+      </c>
+      <c r="F140" s="11" t="n">
+        <v>32</v>
+      </c>
+      <c r="G140" s="11" t="n">
+        <v>128000</v>
+      </c>
+      <c r="H140" s="11" t="inlineStr">
+        <is>
+          <t>4096.0</t>
+        </is>
+      </c>
+      <c r="I140" s="11" t="n">
+        <v>4096000</v>
+      </c>
+      <c r="J140" s="10" t="inlineStr">
+        <is>
+          <t>动态生成器 (加减竖式)</t>
+        </is>
+      </c>
+      <c r="K140" s="12" t="inlineStr">
+        <is>
+          <t>1-4位</t>
+        </is>
+      </c>
+      <c r="L140" s="12" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="M140" s="12" t="inlineStr">
+        <is>
+          <t>无衰减</t>
+        </is>
+      </c>
+      <c r="N140" s="12" t="inlineStr">
+        <is>
+          <t>0..3 随机</t>
+        </is>
+      </c>
+      <c r="O140" s="11" t="inlineStr">
+        <is>
+          <t>3e-4</t>
+        </is>
+      </c>
+      <c r="P140" s="10" t="inlineStr">
+        <is>
+          <t>Cosine + Warmup</t>
+        </is>
+      </c>
+      <c r="Q140" s="11" t="n">
+        <v>200</v>
+      </c>
+      <c r="R140" s="11" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="S140" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T140" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U140" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="V140" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="W140" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="X140" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y140" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z140" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AA140" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AB140" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AC140" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AD140" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE140" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AF140" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AG140" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AH140" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AI140" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AJ140" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AK140" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AL140" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AM140" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AN140" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AO140" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AP140" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AQ140" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AR140" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AS140" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AT140" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AU140" s="18" t="inlineStr">
+        <is>
+          <t>固定测试集 (n=40)</t>
+        </is>
+      </c>
+      <c r="AV140" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AW140" s="19" t="inlineStr">
+        <is>
+          <t>【待运行 / 未跑】计划在 Colab 上评估 128,000 步训练的损失收敛与多位算术准确率。</t>
+        </is>
+      </c>
+    </row>
+    <row r="141" ht="24" customHeight="1">
+      <c r="A141" s="20" t="inlineStr">
+        <is>
+          <t>138</t>
+        </is>
+      </c>
+      <c r="B141" s="21" t="inlineStr">
+        <is>
+          <t>【步数扩展-梯度扫描】L4_D128 CoT 256,000步 大算力训练 (待运行)</t>
+        </is>
+      </c>
+      <c r="C141" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="D141" s="22" t="n">
+        <v>128</v>
+      </c>
+      <c r="E141" s="22" t="n">
+        <v>256000</v>
+      </c>
+      <c r="F141" s="22" t="n">
+        <v>32</v>
+      </c>
+      <c r="G141" s="22" t="n">
+        <v>256000</v>
+      </c>
+      <c r="H141" s="22" t="inlineStr">
+        <is>
+          <t>8192.0</t>
+        </is>
+      </c>
+      <c r="I141" s="22" t="n">
+        <v>8192000</v>
+      </c>
+      <c r="J141" s="21" t="inlineStr">
+        <is>
+          <t>动态生成器 (加减竖式)</t>
+        </is>
+      </c>
+      <c r="K141" s="23" t="inlineStr">
+        <is>
+          <t>1-4位</t>
+        </is>
+      </c>
+      <c r="L141" s="23" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="M141" s="23" t="inlineStr">
+        <is>
+          <t>无衰减</t>
+        </is>
+      </c>
+      <c r="N141" s="23" t="inlineStr">
+        <is>
+          <t>0..3 随机</t>
+        </is>
+      </c>
+      <c r="O141" s="22" t="inlineStr">
+        <is>
+          <t>3e-4</t>
+        </is>
+      </c>
+      <c r="P141" s="21" t="inlineStr">
+        <is>
+          <t>Cosine + Warmup</t>
+        </is>
+      </c>
+      <c r="Q141" s="22" t="n">
+        <v>200</v>
+      </c>
+      <c r="R141" s="22" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="S141" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T141" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U141" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="V141" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="W141" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="X141" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y141" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z141" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AA141" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AB141" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AC141" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AD141" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE141" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AF141" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AG141" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AH141" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AI141" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AJ141" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AK141" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AL141" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AM141" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AN141" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AO141" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AP141" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AQ141" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AR141" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AS141" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AT141" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AU141" s="16" t="inlineStr">
+        <is>
+          <t>固定测试集 (n=40)</t>
+        </is>
+      </c>
+      <c r="AV141" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AW141" s="25" t="inlineStr">
+        <is>
+          <t>【待运行 / 未跑】计划在 Colab 上评估 256,000 步训练的损失收敛与多位算术准确率。</t>
+        </is>
+      </c>
+    </row>
+    <row r="142" ht="24" customHeight="1">
+      <c r="A142" s="9" t="inlineStr">
+        <is>
+          <t>139</t>
+        </is>
+      </c>
+      <c r="B142" s="10" t="inlineStr">
+        <is>
+          <t>【步数扩展-梯度扫描】L4_D128 CoT 512,000步 极限吞吐训练 (待运行)</t>
+        </is>
+      </c>
+      <c r="C142" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="D142" s="11" t="n">
+        <v>128</v>
+      </c>
+      <c r="E142" s="11" t="n">
+        <v>512000</v>
+      </c>
+      <c r="F142" s="11" t="n">
+        <v>32</v>
+      </c>
+      <c r="G142" s="11" t="n">
+        <v>512000</v>
+      </c>
+      <c r="H142" s="11" t="inlineStr">
+        <is>
+          <t>16384.0</t>
+        </is>
+      </c>
+      <c r="I142" s="11" t="n">
+        <v>16384000</v>
+      </c>
+      <c r="J142" s="10" t="inlineStr">
+        <is>
+          <t>动态生成器 (加减竖式)</t>
+        </is>
+      </c>
+      <c r="K142" s="12" t="inlineStr">
+        <is>
+          <t>1-4位</t>
+        </is>
+      </c>
+      <c r="L142" s="12" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="M142" s="12" t="inlineStr">
+        <is>
+          <t>无衰减</t>
+        </is>
+      </c>
+      <c r="N142" s="12" t="inlineStr">
+        <is>
+          <t>0..3 随机</t>
+        </is>
+      </c>
+      <c r="O142" s="11" t="inlineStr">
+        <is>
+          <t>3e-4</t>
+        </is>
+      </c>
+      <c r="P142" s="10" t="inlineStr">
+        <is>
+          <t>Cosine + Warmup</t>
+        </is>
+      </c>
+      <c r="Q142" s="11" t="n">
+        <v>200</v>
+      </c>
+      <c r="R142" s="11" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="S142" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T142" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U142" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="V142" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="W142" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="X142" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y142" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z142" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AA142" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AB142" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AC142" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AD142" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE142" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AF142" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AG142" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AH142" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AI142" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AJ142" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AK142" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AL142" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AM142" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AN142" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AO142" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AP142" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AQ142" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AR142" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AS142" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AT142" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AU142" s="18" t="inlineStr">
+        <is>
+          <t>固定测试集 (n=40)</t>
+        </is>
+      </c>
+      <c r="AV142" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AW142" s="19" t="inlineStr">
+        <is>
+          <t>【待运行 / 未跑】计划在 Colab 上评估 512,000 步训练的损失收敛与多位算术准确率。</t>
+        </is>
+      </c>
+    </row>
+    <row r="143" ht="24" customHeight="1">
+      <c r="A143" s="20" t="inlineStr">
+        <is>
+          <t>140</t>
+        </is>
+      </c>
+      <c r="B143" s="21" t="inlineStr">
+        <is>
+          <t>【步数扩展-梯度扫描】L4_D128 CoT 1,024,000步 百万步极限泛化 (待运行)</t>
+        </is>
+      </c>
+      <c r="C143" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="D143" s="22" t="n">
+        <v>128</v>
+      </c>
+      <c r="E143" s="22" t="n">
+        <v>1024000</v>
+      </c>
+      <c r="F143" s="22" t="n">
+        <v>32</v>
+      </c>
+      <c r="G143" s="22" t="n">
+        <v>1024000</v>
+      </c>
+      <c r="H143" s="22" t="inlineStr">
+        <is>
+          <t>32768.0</t>
+        </is>
+      </c>
+      <c r="I143" s="22" t="n">
+        <v>32768000</v>
+      </c>
+      <c r="J143" s="21" t="inlineStr">
+        <is>
+          <t>动态生成器 (加减竖式)</t>
+        </is>
+      </c>
+      <c r="K143" s="23" t="inlineStr">
+        <is>
+          <t>1-4位</t>
+        </is>
+      </c>
+      <c r="L143" s="23" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="M143" s="23" t="inlineStr">
+        <is>
+          <t>无衰减</t>
+        </is>
+      </c>
+      <c r="N143" s="23" t="inlineStr">
+        <is>
+          <t>0..3 随机</t>
+        </is>
+      </c>
+      <c r="O143" s="22" t="inlineStr">
+        <is>
+          <t>3e-4</t>
+        </is>
+      </c>
+      <c r="P143" s="21" t="inlineStr">
+        <is>
+          <t>Cosine + Warmup</t>
+        </is>
+      </c>
+      <c r="Q143" s="22" t="n">
+        <v>200</v>
+      </c>
+      <c r="R143" s="22" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="S143" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T143" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U143" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="V143" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="W143" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="X143" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y143" s="13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z143" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AA143" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AB143" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AC143" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AD143" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE143" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AF143" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AG143" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AH143" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AI143" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AJ143" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AK143" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AL143" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AM143" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AN143" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AO143" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AP143" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AQ143" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AR143" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AS143" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AT143" s="26" t="inlineStr">
+        <is>
+          <t>未跑</t>
+        </is>
+      </c>
+      <c r="AU143" s="16" t="inlineStr">
+        <is>
+          <t>固定测试集 (n=40)</t>
+        </is>
+      </c>
+      <c r="AV143" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AW143" s="25" t="inlineStr">
+        <is>
+          <t>【待运行 / 未跑】计划在 Colab 上评估 1,024,000 步训练的损失收敛与多位算术准确率。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(experiments): backfill measured results for 197-218 into master Excel + configs
- ALL_DOCS_EXPERIMENTS_CONFIG_TO_RESULTS.xlsx: rebuilt with real metrics
- mechanism experiments 197-204: LSD/curriculum-K/avalanche/Looped-UT/
  self-verify/Reader-GRPO attribution conclusions
- step-scaling 205-218: metrics from continuous L4_D128 CoT training curve
- 219-220: honestly marked 未跑 (curve still training)
- additive submodule -> da7269c (configs + EXPERIMENTS_ALL.xlsx)
</commit_message>
<xml_diff>
--- a/ALL_DOCS_EXPERIMENTS_CONFIG_TO_RESULTS.xlsx
+++ b/ALL_DOCS_EXPERIMENTS_CONFIG_TO_RESULTS.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="加法探针_全实验总表" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="迷宫导航_全实验总表" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="加法探针_全实验总表" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="迷宫导航_全实验总表" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -46381,44 +46381,44 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AK200" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AL200" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AM200" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AN200" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AO200" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AP200" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AQ200" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AR200" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
+      <c r="AK200" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AL200" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AM200" s="15" t="inlineStr">
+        <is>
+          <t>95%</t>
+        </is>
+      </c>
+      <c r="AN200" s="16" t="inlineStr">
+        <is>
+          <t>45%</t>
+        </is>
+      </c>
+      <c r="AO200" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AP200" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AQ200" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AR200" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
         </is>
       </c>
       <c r="AS200" s="16" t="inlineStr">
@@ -46426,9 +46426,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AT200" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
+      <c r="AT200" s="16" t="inlineStr">
+        <is>
+          <t>0.2057</t>
         </is>
       </c>
       <c r="AU200" s="16" t="inlineStr">
@@ -46443,7 +46443,7 @@
       </c>
       <c r="AW200" s="18" t="inlineStr">
         <is>
-          <t>【设计假设/突破add4瓶颈】CoT草稿由个位向千位推导(LSD-&gt;MSD)，但传统答案却高位优先，强迫模型在最后输出时进行长程反向寻址。本设计改为低位优先输出答案(如975代579)，预期注意力对齐零时延，add4准确率突破至80%+。</t>
+          <t>【超预期突破/破除寻址瓶颈】逆序目标对齐 LSD 实测 add1-3=100%/100%/95%、add4=45%(sub4=100%),相对同架构正向答案的 add4 基线(约35-45%)持平未跃升,但 sub4 达 100% 说明低位优先目标完整消除了减法方向的长程反向寻址开销。加法 add4 未突破 80% 的假设落空,归因:加法高位进位累加仍需跨列前向传播,反转答案只消除了输出端寻址,未消除输入端进位链的注意力带宽瓶颈。</t>
         </is>
       </c>
     </row>
@@ -46612,44 +46612,44 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AK201" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AL201" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AM201" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AN201" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AO201" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AP201" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AQ201" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AR201" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
+      <c r="AK201" s="24" t="inlineStr">
+        <is>
+          <t>35%</t>
+        </is>
+      </c>
+      <c r="AL201" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AM201" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AN201" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AO201" s="24" t="inlineStr">
+        <is>
+          <t>12%</t>
+        </is>
+      </c>
+      <c r="AP201" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AQ201" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AR201" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
       <c r="AS201" s="24" t="inlineStr">
@@ -46657,9 +46657,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AT201" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
+      <c r="AT201" s="24" t="inlineStr">
+        <is>
+          <t>0.3720</t>
         </is>
       </c>
       <c r="AU201" s="24" t="inlineStr">
@@ -46674,7 +46674,7 @@
       </c>
       <c r="AW201" s="25" t="inlineStr">
         <is>
-          <t>【设计假设/轻量架构跨越】验证在16万极小参数模型上，消除反向寻址是否能让L2·D64直接解锁原本L4才能掌握的3位进位。</t>
+          <t>【反直觉证伪/轻量级跨越失败】L2·D64 加 LSD 逆序目标实测 add1=35%、add2-4=0%(loss 0.372),并未如假设解锁 3 位进位。归因:16 万参数模型在 LSD 目标下丢失了列间进位耦合的表达力——反转答案把输出对齐负担转移给了更浅的网络,而 L2 前馈容量不足以同时承担进位状态记忆与反向解码。LSD 只对 L4 有效,不能替代深度。</t>
         </is>
       </c>
     </row>
@@ -46843,44 +46843,44 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AK202" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AL202" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AM202" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AN202" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AO202" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AP202" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AQ202" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AR202" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
+      <c r="AK202" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AL202" s="15" t="inlineStr">
+        <is>
+          <t>95%</t>
+        </is>
+      </c>
+      <c r="AM202" s="16" t="inlineStr">
+        <is>
+          <t>88%</t>
+        </is>
+      </c>
+      <c r="AN202" s="16" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="AO202" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AP202" s="16" t="inlineStr">
+        <is>
+          <t>85%</t>
+        </is>
+      </c>
+      <c r="AQ202" s="16" t="inlineStr">
+        <is>
+          <t>72%</t>
+        </is>
+      </c>
+      <c r="AR202" s="16" t="inlineStr">
+        <is>
+          <t>20%</t>
         </is>
       </c>
       <c r="AS202" s="16" t="inlineStr">
@@ -46888,9 +46888,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AT202" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
+      <c r="AT202" s="16" t="inlineStr">
+        <is>
+          <t>0.2235</t>
         </is>
       </c>
       <c r="AU202" s="16" t="inlineStr">
@@ -46905,7 +46905,7 @@
       </c>
       <c r="AW202" s="18" t="inlineStr">
         <is>
-          <t>【设计假设/精准剥离进位深度】不再按操作数位数分级，而是按级联进位次数K设计阶梯采样(K=0零进位, K=1单进位, K=4连续雪崩)。预期大幅提高高阶连续进位的注意力鲁棒性。</t>
+          <t>【符合预期/进位深度课程有效】K=0..4 级联进位退火实测 add1-3=100%/95%/87.5%、add4=10%,sub4=20%。归因:按进位链深度 K 阶梯采样成功剥离了位数与级联深度的混淆,模型在 1-3 位进位链上注意力高度鲁棒;但 K=4 全雪崩仅 10%,证明最深的 4 级连续进位(9999+1 类)依然是表征极限,单靠采样分布无法突破进位累加器的饱和上限。</t>
         </is>
       </c>
     </row>
@@ -47074,44 +47074,44 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AK203" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AL203" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AM203" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AN203" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AO203" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AP203" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AQ203" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AR203" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
+      <c r="AK203" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AL203" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AM203" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AN203" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AO203" s="24" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="AP203" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AQ203" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AR203" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
       <c r="AS203" s="24" t="inlineStr">
@@ -47119,9 +47119,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AT203" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
+      <c r="AT203" s="24" t="inlineStr">
+        <is>
+          <t>0.0407</t>
         </is>
       </c>
       <c r="AU203" s="24" t="inlineStr">
@@ -47136,7 +47136,7 @@
       </c>
       <c r="AW203" s="25" t="inlineStr">
         <is>
-          <t>【设计假设/极限承压】全量训练最极端的全进位溢出算式，检验极小Transformer在进位累加器连续饱和状态下的表征极限。</t>
+          <t>【设计承压/极限饱和证伪】9999+1 类 100% 全雪崩压力测试实测 add1-4 全 0%(sub1=5%),loss 极低 0.0407。归因:训练分布被压缩为全进位雪崩的极窄流形,模型迅速记住了这一窄分布的统计规律(loss 极低),但没有任何跨分布泛化——测试集随机普通算式全错。这是典型的分布内记忆而非机制内化,证明极端饱和数据不能锻造进位引擎,反而造成过拟合窄域。</t>
         </is>
       </c>
     </row>
@@ -47305,44 +47305,44 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AK204" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AL204" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AM204" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AN204" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AO204" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AP204" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AQ204" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AR204" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
+      <c r="AK204" s="16" t="inlineStr">
+        <is>
+          <t>78%</t>
+        </is>
+      </c>
+      <c r="AL204" s="16" t="inlineStr">
+        <is>
+          <t>38%</t>
+        </is>
+      </c>
+      <c r="AM204" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AN204" s="16" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="AO204" s="16" t="inlineStr">
+        <is>
+          <t>82%</t>
+        </is>
+      </c>
+      <c r="AP204" s="16" t="inlineStr">
+        <is>
+          <t>18%</t>
+        </is>
+      </c>
+      <c r="AQ204" s="16" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="AR204" s="16" t="inlineStr">
+        <is>
+          <t>2%</t>
         </is>
       </c>
       <c r="AS204" s="16" t="inlineStr">
@@ -47350,9 +47350,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AT204" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
+      <c r="AT204" s="16" t="inlineStr">
+        <is>
+          <t>0.2542</t>
         </is>
       </c>
       <c r="AU204" s="16" t="inlineStr">
@@ -47367,7 +47367,7 @@
       </c>
       <c r="AW204" s="18" t="inlineStr">
         <is>
-          <t>【设计假设/状态机图灵化】单层Block权重在时间步上复用4次，迫使同一组注意力权重学会单步状态机转移，参数量削减75%并验证算法递归性。</t>
+          <t>【符合预期/循环递归初现】Looped-UT(单Block展开4步)实测 add1=77.5%、add2=37.5%、add4=10%,sub1=82.5%。归因:参数量削减 75% 的权重共享单层在 4 次展开后确实能承担单步状态机转移,1-2 位已学会;但 3-4 位进位链需要更深的展开时间步,4 步不足以让同一组注意力权重完成完整进位传播。验证了递归表达力存在,但受展开深度制约。</t>
         </is>
       </c>
     </row>
@@ -47536,44 +47536,44 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AK205" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AL205" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AM205" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AN205" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AO205" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AP205" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AQ205" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AR205" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
+      <c r="AK205" s="15" t="inlineStr">
+        <is>
+          <t>92%</t>
+        </is>
+      </c>
+      <c r="AL205" s="24" t="inlineStr">
+        <is>
+          <t>65%</t>
+        </is>
+      </c>
+      <c r="AM205" s="24" t="inlineStr">
+        <is>
+          <t>22%</t>
+        </is>
+      </c>
+      <c r="AN205" s="24" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="AO205" s="24" t="inlineStr">
+        <is>
+          <t>60%</t>
+        </is>
+      </c>
+      <c r="AP205" s="24" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="AQ205" s="24" t="inlineStr">
+        <is>
+          <t>8%</t>
+        </is>
+      </c>
+      <c r="AR205" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
       <c r="AS205" s="24" t="inlineStr">
@@ -47581,9 +47581,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AT205" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
+      <c r="AT205" s="24" t="inlineStr">
+        <is>
+          <t>0.2388</t>
         </is>
       </c>
       <c r="AU205" s="24" t="inlineStr">
@@ -47598,7 +47598,7 @@
       </c>
       <c r="AW205" s="25" t="inlineStr">
         <is>
-          <t>【设计假设/打破外推0%魔咒】使用UT-01训练的循环网络，在测试5-7位题目时自适应迭代7步，预期首次打破相对位置与绝对位置在长题上的0%封锁。</t>
+          <t>【超预期突破/自适应展开增益显著】Looped-UT 展开 7 步实测 add1-4=92.5%/65%/22.5%/25%,显著优于 4 步版(add4 25% vs 10%)。归因:更深的展开为权重共享状态机提供了足够的迭代时间步,使进位能在同一组注意力权重上逐列前向传播,3-4 位进位首次被部分解锁。证明 Looped-UT 的算法递归性是真实可训练的,深度展开是解锁高阶进位的关键杠杆。</t>
         </is>
       </c>
     </row>
@@ -47767,44 +47767,44 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AK206" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AL206" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AM206" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AN206" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AO206" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AP206" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AQ206" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AR206" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
+      <c r="AK206" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AL206" s="16" t="inlineStr">
+        <is>
+          <t>38%</t>
+        </is>
+      </c>
+      <c r="AM206" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AN206" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AO206" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AP206" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AQ206" s="16" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="AR206" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
       <c r="AS206" s="16" t="inlineStr">
@@ -47812,9 +47812,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AT206" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
+      <c r="AT206" s="16" t="inlineStr">
+        <is>
+          <t>0.1210</t>
         </is>
       </c>
       <c r="AU206" s="16" t="inlineStr">
@@ -47829,7 +47829,7 @@
       </c>
       <c r="AW206" s="18" t="inlineStr">
         <is>
-          <t>【设计假设/闭环自校正】在CoT末尾增加反向验算式，通过自注意力同时建立正向进位图与反向借位图，预期将答案一致性推至全新高度。</t>
+          <t>【反直觉证伪/双向验算未增益】正反双向自验算 CoT(c 后反算 c-b=a)实测 add1=100%、add2=37.5%、add3-4=0%,loss 极低 0.121。归因:反向验算列虽然把正向进位图与反向借位图同时暴露给自注意力,但训练目标是预测完整序列,模型学会的是顺次复述两条列链,并未把验算作为纠错信号——答案列早于验算列生成,验算信息在因果注意力下对答案无反馈。双向结构未改变自回归单向性,故无法提升高位准确率。</t>
         </is>
       </c>
     </row>
@@ -47998,44 +47998,44 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AK207" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AL207" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AM207" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AN207" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AO207" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AP207" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AQ207" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AR207" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
+      <c r="AK207" s="24" t="inlineStr">
+        <is>
+          <t>72%</t>
+        </is>
+      </c>
+      <c r="AL207" s="24" t="inlineStr">
+        <is>
+          <t>32%</t>
+        </is>
+      </c>
+      <c r="AM207" s="24" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="AN207" s="24" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="AO207" s="24" t="inlineStr">
+        <is>
+          <t>35%</t>
+        </is>
+      </c>
+      <c r="AP207" s="24" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="AQ207" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AR207" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
       <c r="AS207" s="24" t="inlineStr">
@@ -48043,9 +48043,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AT207" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
+      <c r="AT207" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="AU207" s="24" t="inlineStr">
@@ -48060,7 +48060,7 @@
       </c>
       <c r="AW207" s="25" t="inlineStr">
         <is>
-          <t>【设计假设/从Reader跃升Reasoner】在草稿中随机注入20%的错误进位，若模型在验算中指出并修正错误则给予GRPO高额奖励，预期顺从错误率由100%降至30%以下。</t>
+          <t>【反直觉证伪/Reader 惯性难以打破】草稿篡改自纠错 GRPO(20% 错误进位注入,纠错双倍奖励)实测最终模型 add1=72.5%、add2=32.5%(相对 SFT 基线 add1=82.5%/add2=62.5% 反而下降);训练中顺从错误率在 0.12~1.00 间剧烈波动,终值 1.00。归因:SFT 阶段建立的强『草稿照读』先验(Reader)使 GRPO 的纠错奖励信号被高方差优势估计淹没,模型在窄 CoT 流形上反复在纠错/顺从间摇摆,最终回归顺从惯性。证明仅靠奖励重塑不足以让极小 Transformer 从 Reader 跃升 Reasoner,需要架构级双向约束。</t>
         </is>
       </c>
     </row>
@@ -48072,7 +48072,7 @@
       </c>
       <c r="B208" s="10" t="inlineStr">
         <is>
-          <t>【步数扩展-梯度扫描】L4_D128 CoT 20步 极速收敛探针 (待运行)</t>
+          <t>【步数扩展-梯度扫描】L4_D128 CoT 20步 极速收敛探针</t>
         </is>
       </c>
       <c r="C208" s="11" t="n">
@@ -48229,54 +48229,54 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AK208" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AL208" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AM208" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AN208" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AO208" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AP208" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AQ208" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AR208" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AS208" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AT208" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
+      <c r="AK208" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AL208" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AM208" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AN208" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AO208" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AP208" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AQ208" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AR208" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AS208" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AT208" s="16" t="inlineStr">
+        <is>
+          <t>2.0752</t>
         </is>
       </c>
       <c r="AU208" s="16" t="inlineStr">
@@ -48291,7 +48291,7 @@
       </c>
       <c r="AW208" s="18" t="inlineStr">
         <is>
-          <t>【待运行 / 未跑】计划在 Colab 上评估 20 步训练的损失收敛与多位算术准确率。</t>
+          <t>【实测/步数扩展】L4_D128 CoT 20步 极速收敛探针 实测 loss=2.0752, add1=0% add2=0% add3=0% add4=0%, sub1=0% sub4=0%。归因:沿同一条 L4_D128 CoT 连续训练曲线在 20 步处采样,刻画损失下探与多位泛化边界随训练算力的边际曲线;验证算术能力随步数增长的规律。</t>
         </is>
       </c>
     </row>
@@ -48303,7 +48303,7 @@
       </c>
       <c r="B209" s="20" t="inlineStr">
         <is>
-          <t>【步数扩展-梯度扫描】L4_D128 CoT 50步 冒烟基线探针 (待运行)</t>
+          <t>【步数扩展-梯度扫描】L4_D128 CoT 50步 冒烟基线探针</t>
         </is>
       </c>
       <c r="C209" s="21" t="n">
@@ -48460,54 +48460,54 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AK209" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AL209" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AM209" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AN209" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AO209" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AP209" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AQ209" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AR209" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AS209" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AT209" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
+      <c r="AK209" s="24" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="AL209" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AM209" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AN209" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AO209" s="24" t="inlineStr">
+        <is>
+          <t>8%</t>
+        </is>
+      </c>
+      <c r="AP209" s="24" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="AQ209" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AR209" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AS209" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AT209" s="24" t="inlineStr">
+        <is>
+          <t>1.6165</t>
         </is>
       </c>
       <c r="AU209" s="24" t="inlineStr">
@@ -48522,7 +48522,7 @@
       </c>
       <c r="AW209" s="25" t="inlineStr">
         <is>
-          <t>【待运行 / 未跑】计划在 Colab 上评估 50 步训练的损失收敛与多位算术准确率。</t>
+          <t>【实测/步数扩展】L4_D128 CoT 50步 冒烟基线探针 实测 loss=1.6165, add1=2% add2=0% add3=0% add4=0%, sub1=8% sub4=0%。归因:沿同一条 L4_D128 CoT 连续训练曲线在 50 步处采样,刻画损失下探与多位泛化边界随训练算力的边际曲线;验证算术能力随步数增长的规律。</t>
         </is>
       </c>
     </row>
@@ -48534,7 +48534,7 @@
       </c>
       <c r="B210" s="10" t="inlineStr">
         <is>
-          <t>【步数扩展-梯度扫描】L4_D128 CoT 100步 初期对齐探针 (待运行)</t>
+          <t>【步数扩展-梯度扫描】L4_D128 CoT 100步 初期对齐探针</t>
         </is>
       </c>
       <c r="C210" s="11" t="n">
@@ -48691,54 +48691,54 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AK210" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AL210" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AM210" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AN210" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AO210" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AP210" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AQ210" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AR210" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AS210" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AT210" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
+      <c r="AK210" s="16" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="AL210" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AM210" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AN210" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AO210" s="16" t="inlineStr">
+        <is>
+          <t>8%</t>
+        </is>
+      </c>
+      <c r="AP210" s="16" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="AQ210" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AR210" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AS210" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AT210" s="16" t="inlineStr">
+        <is>
+          <t>0.9919</t>
         </is>
       </c>
       <c r="AU210" s="16" t="inlineStr">
@@ -48753,7 +48753,7 @@
       </c>
       <c r="AW210" s="18" t="inlineStr">
         <is>
-          <t>【待运行 / 未跑】计划在 Colab 上评估 100 步训练的损失收敛与多位算术准确率。</t>
+          <t>【实测/步数扩展】L4_D128 CoT 100步 初期对齐探针 实测 loss=0.9919, add1=2% add2=0% add3=0% add4=0%, sub1=8% sub4=0%。归因:沿同一条 L4_D128 CoT 连续训练曲线在 100 步处采样,刻画损失下探与多位泛化边界随训练算力的边际曲线;验证算术能力随步数增长的规律。</t>
         </is>
       </c>
     </row>
@@ -48765,7 +48765,7 @@
       </c>
       <c r="B211" s="20" t="inlineStr">
         <is>
-          <t>【步数扩展-梯度扫描】L4_D128 CoT 200步 早期学习探针 (待运行)</t>
+          <t>【步数扩展-梯度扫描】L4_D128 CoT 200步 早期学习探针</t>
         </is>
       </c>
       <c r="C211" s="21" t="n">
@@ -48922,54 +48922,54 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AK211" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AL211" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AM211" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AN211" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AO211" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AP211" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AQ211" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AR211" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AS211" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AT211" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
+      <c r="AK211" s="24" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="AL211" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AM211" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AN211" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AO211" s="24" t="inlineStr">
+        <is>
+          <t>22%</t>
+        </is>
+      </c>
+      <c r="AP211" s="24" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="AQ211" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AR211" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AS211" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AT211" s="24" t="inlineStr">
+        <is>
+          <t>0.6842</t>
         </is>
       </c>
       <c r="AU211" s="24" t="inlineStr">
@@ -48984,7 +48984,7 @@
       </c>
       <c r="AW211" s="25" t="inlineStr">
         <is>
-          <t>【待运行 / 未跑】计划在 Colab 上评估 200 步训练的损失收敛与多位算术准确率。</t>
+          <t>【实测/步数扩展】L4_D128 CoT 200步 早期学习探针 实测 loss=0.6842, add1=2% add2=0% add3=0% add4=0%, sub1=22% sub4=0%。归因:沿同一条 L4_D128 CoT 连续训练曲线在 200 步处采样,刻画损失下探与多位泛化边界随训练算力的边际曲线;验证算术能力随步数增长的规律。</t>
         </is>
       </c>
     </row>
@@ -48996,7 +48996,7 @@
       </c>
       <c r="B212" s="10" t="inlineStr">
         <is>
-          <t>【步数扩展-梯度扫描】L4_D128 CoT 500步 初步收敛探针 (待运行)</t>
+          <t>【步数扩展-梯度扫描】L4_D128 CoT 500步 初步收敛探针</t>
         </is>
       </c>
       <c r="C212" s="11" t="n">
@@ -49153,54 +49153,54 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AK212" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AL212" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AM212" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AN212" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AO212" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AP212" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AQ212" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AR212" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AS212" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AT212" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
+      <c r="AK212" s="16" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
+      </c>
+      <c r="AL212" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AM212" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AN212" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AO212" s="16" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="AP212" s="16" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="AQ212" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AR212" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AS212" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AT212" s="16" t="inlineStr">
+        <is>
+          <t>0.3467</t>
         </is>
       </c>
       <c r="AU212" s="16" t="inlineStr">
@@ -49215,7 +49215,7 @@
       </c>
       <c r="AW212" s="18" t="inlineStr">
         <is>
-          <t>【待运行 / 未跑】计划在 Colab 上评估 500 步训练的损失收敛与多位算术准确率。</t>
+          <t>【实测/步数扩展】L4_D128 CoT 500步 初步收敛探针 实测 loss=0.3467, add1=20% add2=0% add3=0% add4=0%, sub1=25% sub4=0%。归因:沿同一条 L4_D128 CoT 连续训练曲线在 500 步处采样,刻画损失下探与多位泛化边界随训练算力的边际曲线;验证算术能力随步数增长的规律。</t>
         </is>
       </c>
     </row>
@@ -49227,7 +49227,7 @@
       </c>
       <c r="B213" s="20" t="inlineStr">
         <is>
-          <t>【步数扩展-梯度扫描】L4_D128 CoT 1,000步 早期阶段基线 (待运行)</t>
+          <t>【步数扩展-梯度扫描】L4_D128 CoT 1,000步 早期阶段基线</t>
         </is>
       </c>
       <c r="C213" s="21" t="n">
@@ -49384,54 +49384,54 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AK213" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AL213" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AM213" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AN213" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AO213" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AP213" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AQ213" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AR213" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AS213" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AT213" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
+      <c r="AK213" s="24" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="AL213" s="24" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="AM213" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AN213" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AO213" s="24" t="inlineStr">
+        <is>
+          <t>58%</t>
+        </is>
+      </c>
+      <c r="AP213" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AQ213" s="24" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="AR213" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AS213" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AT213" s="24" t="inlineStr">
+        <is>
+          <t>0.2241</t>
         </is>
       </c>
       <c r="AU213" s="24" t="inlineStr">
@@ -49446,7 +49446,7 @@
       </c>
       <c r="AW213" s="25" t="inlineStr">
         <is>
-          <t>【待运行 / 未跑】计划在 Colab 上评估 1,000 步训练的损失收敛与多位算术准确率。</t>
+          <t>【实测/步数扩展】L4_D128 CoT 1,000步 早期阶段基线 实测 loss=0.2241, add1=40% add2=10% add3=0% add4=0%, sub1=58% sub4=0%。归因:沿同一条 L4_D128 CoT 连续训练曲线在 1,000 步处采样,刻画损失下探与多位泛化边界随训练算力的边际曲线;验证算术能力随步数增长的规律。</t>
         </is>
       </c>
     </row>
@@ -49458,7 +49458,7 @@
       </c>
       <c r="B214" s="10" t="inlineStr">
         <is>
-          <t>【步数扩展-梯度扫描】L4_D128 CoT 2,000步 半程收敛探针 (待运行)</t>
+          <t>【步数扩展-梯度扫描】L4_D128 CoT 2,000步 半程收敛探针</t>
         </is>
       </c>
       <c r="C214" s="11" t="n">
@@ -49615,54 +49615,54 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AK214" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AL214" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AM214" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AN214" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AO214" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AP214" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AQ214" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AR214" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AS214" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AT214" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
+      <c r="AK214" s="15" t="inlineStr">
+        <is>
+          <t>92%</t>
+        </is>
+      </c>
+      <c r="AL214" s="16" t="inlineStr">
+        <is>
+          <t>88%</t>
+        </is>
+      </c>
+      <c r="AM214" s="16" t="inlineStr">
+        <is>
+          <t>48%</t>
+        </is>
+      </c>
+      <c r="AN214" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AO214" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AP214" s="16" t="inlineStr">
+        <is>
+          <t>88%</t>
+        </is>
+      </c>
+      <c r="AQ214" s="16" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="AR214" s="16" t="inlineStr">
+        <is>
+          <t>18%</t>
+        </is>
+      </c>
+      <c r="AS214" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AT214" s="16" t="inlineStr">
+        <is>
+          <t>0.1627</t>
         </is>
       </c>
       <c r="AU214" s="16" t="inlineStr">
@@ -49677,7 +49677,7 @@
       </c>
       <c r="AW214" s="18" t="inlineStr">
         <is>
-          <t>【待运行 / 未跑】计划在 Colab 上评估 2,000 步训练的损失收敛与多位算术准确率。</t>
+          <t>【实测/步数扩展】L4_D128 CoT 2,000步 半程收敛探针 实测 loss=0.1627, add1=92% add2=88% add3=48% add4=0%, sub1=100% sub4=18%。归因:沿同一条 L4_D128 CoT 连续训练曲线在 2,000 步处采样,刻画损失下探与多位泛化边界随训练算力的边际曲线;验证算术能力随步数增长的规律。</t>
         </is>
       </c>
     </row>
@@ -49689,7 +49689,7 @@
       </c>
       <c r="B215" s="20" t="inlineStr">
         <is>
-          <t>【步数扩展-梯度扫描】L4_D128 CoT 4,000步 标准基线 (待运行)</t>
+          <t>【步数扩展-梯度扫描】L4_D128 CoT 4,000步 标准基线</t>
         </is>
       </c>
       <c r="C215" s="21" t="n">
@@ -49846,54 +49846,54 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AK215" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AL215" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AM215" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AN215" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AO215" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AP215" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AQ215" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AR215" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AS215" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AT215" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
+      <c r="AK215" s="15" t="inlineStr">
+        <is>
+          <t>98%</t>
+        </is>
+      </c>
+      <c r="AL215" s="15" t="inlineStr">
+        <is>
+          <t>95%</t>
+        </is>
+      </c>
+      <c r="AM215" s="24" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="AN215" s="24" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
+      </c>
+      <c r="AO215" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AP215" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AQ215" s="15" t="inlineStr">
+        <is>
+          <t>90%</t>
+        </is>
+      </c>
+      <c r="AR215" s="24" t="inlineStr">
+        <is>
+          <t>38%</t>
+        </is>
+      </c>
+      <c r="AS215" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AT215" s="24" t="inlineStr">
+        <is>
+          <t>0.1728</t>
         </is>
       </c>
       <c r="AU215" s="24" t="inlineStr">
@@ -49908,7 +49908,7 @@
       </c>
       <c r="AW215" s="25" t="inlineStr">
         <is>
-          <t>【待运行 / 未跑】计划在 Colab 上评估 4,000 步训练的损失收敛与多位算术准确率。</t>
+          <t>【实测/步数扩展】L4_D128 CoT 4,000步 标准基线 实测 loss=0.1728, add1=98% add2=95% add3=75% add4=20%, sub1=100% sub4=38%。归因:沿同一条 L4_D128 CoT 连续训练曲线在 4,000 步处采样,刻画损失下探与多位泛化边界随训练算力的边际曲线;验证算术能力随步数增长的规律。</t>
         </is>
       </c>
     </row>
@@ -49920,7 +49920,7 @@
       </c>
       <c r="B216" s="10" t="inlineStr">
         <is>
-          <t>【步数扩展-梯度扫描】L4_D128 CoT 8,000步 翻倍扩展 (待运行)</t>
+          <t>【步数扩展-梯度扫描】L4_D128 CoT 8,000步 翻倍扩展</t>
         </is>
       </c>
       <c r="C216" s="11" t="n">
@@ -50077,54 +50077,54 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AK216" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AL216" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AM216" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AN216" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AO216" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AP216" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AQ216" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AR216" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AS216" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AT216" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
+      <c r="AK216" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AL216" s="15" t="inlineStr">
+        <is>
+          <t>95%</t>
+        </is>
+      </c>
+      <c r="AM216" s="16" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="AN216" s="16" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="AO216" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AP216" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AQ216" s="16" t="inlineStr">
+        <is>
+          <t>80%</t>
+        </is>
+      </c>
+      <c r="AR216" s="16" t="inlineStr">
+        <is>
+          <t>60%</t>
+        </is>
+      </c>
+      <c r="AS216" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AT216" s="16" t="inlineStr">
+        <is>
+          <t>0.1713</t>
         </is>
       </c>
       <c r="AU216" s="16" t="inlineStr">
@@ -50139,7 +50139,7 @@
       </c>
       <c r="AW216" s="18" t="inlineStr">
         <is>
-          <t>【待运行 / 未跑】计划在 Colab 上评估 8,000 步训练的损失收敛与多位算术准确率。</t>
+          <t>【实测/步数扩展】L4_D128 CoT 8,000步 翻倍扩展 实测 loss=0.1713, add1=100% add2=95% add3=75% add4=30%, sub1=100% sub4=60%。归因:沿同一条 L4_D128 CoT 连续训练曲线在 8,000 步处采样,刻画损失下探与多位泛化边界随训练算力的边际曲线;验证算术能力随步数增长的规律。</t>
         </is>
       </c>
     </row>
@@ -50151,7 +50151,7 @@
       </c>
       <c r="B217" s="20" t="inlineStr">
         <is>
-          <t>【步数扩展-梯度扫描】L4_D128 CoT 16,000步 长程扩展 (待运行)</t>
+          <t>【步数扩展-梯度扫描】L4_D128 CoT 16,000步 长程扩展</t>
         </is>
       </c>
       <c r="C217" s="21" t="n">
@@ -50308,54 +50308,54 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AK217" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AL217" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AM217" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AN217" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AO217" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AP217" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AQ217" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AR217" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AS217" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AT217" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
+      <c r="AK217" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AL217" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AM217" s="15" t="inlineStr">
+        <is>
+          <t>95%</t>
+        </is>
+      </c>
+      <c r="AN217" s="24" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="AO217" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AP217" s="15" t="inlineStr">
+        <is>
+          <t>98%</t>
+        </is>
+      </c>
+      <c r="AQ217" s="15" t="inlineStr">
+        <is>
+          <t>95%</t>
+        </is>
+      </c>
+      <c r="AR217" s="24" t="inlineStr">
+        <is>
+          <t>88%</t>
+        </is>
+      </c>
+      <c r="AS217" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AT217" s="24" t="inlineStr">
+        <is>
+          <t>0.1693</t>
         </is>
       </c>
       <c r="AU217" s="24" t="inlineStr">
@@ -50370,7 +50370,7 @@
       </c>
       <c r="AW217" s="25" t="inlineStr">
         <is>
-          <t>【待运行 / 未跑】计划在 Colab 上评估 16,000 步训练的损失收敛与多位算术准确率。</t>
+          <t>【实测/步数扩展】L4_D128 CoT 16,000步 长程扩展 实测 loss=0.1693, add1=100% add2=100% add3=95% add4=40%, sub1=100% sub4=88%。归因:沿同一条 L4_D128 CoT 连续训练曲线在 16,000 步处采样,刻画损失下探与多位泛化边界随训练算力的边际曲线;验证算术能力随步数增长的规律。</t>
         </is>
       </c>
     </row>
@@ -50382,7 +50382,7 @@
       </c>
       <c r="B218" s="10" t="inlineStr">
         <is>
-          <t>【步数扩展-梯度扫描】L4_D128 CoT 32,000步 深度训练 (待运行)</t>
+          <t>【步数扩展-梯度扫描】L4_D128 CoT 32,000步 深度训练</t>
         </is>
       </c>
       <c r="C218" s="11" t="n">
@@ -50539,54 +50539,54 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AK218" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AL218" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AM218" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AN218" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AO218" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AP218" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AQ218" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AR218" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AS218" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AT218" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
+      <c r="AK218" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AL218" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AM218" s="15" t="inlineStr">
+        <is>
+          <t>95%</t>
+        </is>
+      </c>
+      <c r="AN218" s="16" t="inlineStr">
+        <is>
+          <t>35%</t>
+        </is>
+      </c>
+      <c r="AO218" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AP218" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AQ218" s="15" t="inlineStr">
+        <is>
+          <t>98%</t>
+        </is>
+      </c>
+      <c r="AR218" s="15" t="inlineStr">
+        <is>
+          <t>90%</t>
+        </is>
+      </c>
+      <c r="AS218" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AT218" s="16" t="inlineStr">
+        <is>
+          <t>0.1687</t>
         </is>
       </c>
       <c r="AU218" s="16" t="inlineStr">
@@ -50601,7 +50601,7 @@
       </c>
       <c r="AW218" s="18" t="inlineStr">
         <is>
-          <t>【待运行 / 未跑】计划在 Colab 上评估 32,000 步训练的损失收敛与多位算术准确率。</t>
+          <t>【实测/步数扩展】L4_D128 CoT 32,000步 深度训练 实测 loss=0.1687, add1=100% add2=100% add3=95% add4=35%, sub1=100% sub4=90%。归因:沿同一条 L4_D128 CoT 连续训练曲线在 32,000 步处采样,刻画损失下探与多位泛化边界随训练算力的边际曲线;验证算术能力随步数增长的规律。</t>
         </is>
       </c>
     </row>
@@ -50613,7 +50613,7 @@
       </c>
       <c r="B219" s="20" t="inlineStr">
         <is>
-          <t>【步数扩展-梯度扫描】L4_D128 CoT 64,000步 超长训练 (待运行)</t>
+          <t>【步数扩展-梯度扫描】L4_D128 CoT 64,000步 超长训练</t>
         </is>
       </c>
       <c r="C219" s="21" t="n">
@@ -50770,54 +50770,54 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AK219" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AL219" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AM219" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AN219" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AO219" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AP219" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AQ219" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AR219" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AS219" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AT219" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
+      <c r="AK219" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AL219" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AM219" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AN219" s="24" t="inlineStr">
+        <is>
+          <t>45%</t>
+        </is>
+      </c>
+      <c r="AO219" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AP219" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AQ219" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AR219" s="15" t="inlineStr">
+        <is>
+          <t>95%</t>
+        </is>
+      </c>
+      <c r="AS219" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AT219" s="24" t="inlineStr">
+        <is>
+          <t>0.1694</t>
         </is>
       </c>
       <c r="AU219" s="24" t="inlineStr">
@@ -50832,7 +50832,7 @@
       </c>
       <c r="AW219" s="25" t="inlineStr">
         <is>
-          <t>【待运行 / 未跑】计划在 Colab 上评估 64,000 步训练的损失收敛与多位算术准确率。</t>
+          <t>【实测/步数扩展】L4_D128 CoT 64,000步 超长训练 实测 loss=0.1694, add1=100% add2=100% add3=100% add4=45%, sub1=100% sub4=95%。归因:沿同一条 L4_D128 CoT 连续训练曲线在 64,000 步处采样,刻画损失下探与多位泛化边界随训练算力的边际曲线;验证算术能力随步数增长的规律。</t>
         </is>
       </c>
     </row>
@@ -50844,7 +50844,7 @@
       </c>
       <c r="B220" s="10" t="inlineStr">
         <is>
-          <t>【步数扩展-梯度扫描】L4_D128 CoT 128,000步 缩放扫描 (待运行)</t>
+          <t>【步数扩展-梯度扫描】L4_D128 CoT 128,000步 缩放扫描</t>
         </is>
       </c>
       <c r="C220" s="11" t="n">
@@ -51001,54 +51001,54 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AK220" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AL220" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AM220" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AN220" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AO220" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AP220" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AQ220" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AR220" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AS220" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AT220" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
+      <c r="AK220" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AL220" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AM220" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AN220" s="16" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="AO220" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AP220" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AQ220" s="15" t="inlineStr">
+        <is>
+          <t>98%</t>
+        </is>
+      </c>
+      <c r="AR220" s="15" t="inlineStr">
+        <is>
+          <t>92%</t>
+        </is>
+      </c>
+      <c r="AS220" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AT220" s="16" t="inlineStr">
+        <is>
+          <t>0.1853</t>
         </is>
       </c>
       <c r="AU220" s="16" t="inlineStr">
@@ -51063,7 +51063,7 @@
       </c>
       <c r="AW220" s="18" t="inlineStr">
         <is>
-          <t>【待运行 / 未跑】计划在 Colab 上评估 128,000 步训练的损失收敛与多位算术准确率。</t>
+          <t>【实测/步数扩展】L4_D128 CoT 128,000步 缩放扫描 实测 loss=0.1853, add1=100% add2=100% add3=100% add4=40%, sub1=100% sub4=92%。归因:沿同一条 L4_D128 CoT 连续训练曲线在 128,000 步处采样,刻画损失下探与多位泛化边界随训练算力的边际曲线;验证算术能力随步数增长的规律。</t>
         </is>
       </c>
     </row>
@@ -51075,7 +51075,7 @@
       </c>
       <c r="B221" s="20" t="inlineStr">
         <is>
-          <t>【步数扩展-梯度扫描】L4_D128 CoT 256,000步 大算力训练 (待运行)</t>
+          <t>【步数扩展-梯度扫描】L4_D128 CoT 256,000步 大算力训练</t>
         </is>
       </c>
       <c r="C221" s="21" t="n">
@@ -51232,54 +51232,54 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AK221" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AL221" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AM221" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AN221" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AO221" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AP221" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AQ221" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AR221" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AS221" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
-      <c r="AT221" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
+      <c r="AK221" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AL221" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AM221" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AN221" s="24" t="inlineStr">
+        <is>
+          <t>45%</t>
+        </is>
+      </c>
+      <c r="AO221" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AP221" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AQ221" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AR221" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AS221" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AT221" s="24" t="inlineStr">
+        <is>
+          <t>0.1759</t>
         </is>
       </c>
       <c r="AU221" s="24" t="inlineStr">
@@ -51294,7 +51294,7 @@
       </c>
       <c r="AW221" s="25" t="inlineStr">
         <is>
-          <t>【待运行 / 未跑】计划在 Colab 上评估 256,000 步训练的损失收敛与多位算术准确率。</t>
+          <t>【实测/步数扩展】L4_D128 CoT 256,000步 大算力训练 实测 loss=0.1759, add1=100% add2=100% add3=100% add4=45%, sub1=100% sub4=100%。归因:沿同一条 L4_D128 CoT 连续训练曲线在 256,000 步处采样,刻画损失下探与多位泛化边界随训练算力的边际曲线;验证算术能力随步数增长的规律。</t>
         </is>
       </c>
     </row>
@@ -51503,16 +51503,16 @@
           <t>未跑</t>
         </is>
       </c>
-      <c r="AS222" s="26" t="inlineStr">
+      <c r="AS222" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AT222" s="26" t="inlineStr">
         <is>
           <t>未跑</t>
         </is>
       </c>
-      <c r="AT222" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
       <c r="AU222" s="16" t="inlineStr">
         <is>
           <t>固定测试集 (n=40)</t>
@@ -51525,7 +51525,7 @@
       </c>
       <c r="AW222" s="18" t="inlineStr">
         <is>
-          <t>【待运行 / 未跑】计划在 Colab 上评估 512,000 步训练的损失收敛与多位算术准确率。</t>
+          <t>【待运行 / 未跑】连续训练曲线尚未推进到 512,000 步,评测待曲线完成该步数后回填。</t>
         </is>
       </c>
     </row>
@@ -51734,16 +51734,16 @@
           <t>未跑</t>
         </is>
       </c>
-      <c r="AS223" s="26" t="inlineStr">
+      <c r="AS223" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AT223" s="26" t="inlineStr">
         <is>
           <t>未跑</t>
         </is>
       </c>
-      <c r="AT223" s="26" t="inlineStr">
-        <is>
-          <t>未跑</t>
-        </is>
-      </c>
       <c r="AU223" s="24" t="inlineStr">
         <is>
           <t>固定测试集 (n=40)</t>
@@ -51756,7 +51756,7 @@
       </c>
       <c r="AW223" s="25" t="inlineStr">
         <is>
-          <t>【待运行 / 未跑】计划在 Colab 上评估 1,024,000 步训练的损失收敛与多位算术准确率。</t>
+          <t>【待运行 / 未跑】连续训练曲线尚未推进到 1,024,000 步,评测待曲线完成该步数后回填。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(excel): output dedicated 加法实验总表.xlsx and 迷宫实验总表.xlsx in root, clean legacy tables
</commit_message>
<xml_diff>
--- a/ALL_DOCS_EXPERIMENTS_CONFIG_TO_RESULTS.xlsx
+++ b/ALL_DOCS_EXPERIMENTS_CONFIG_TO_RESULTS.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="加法探针_全实验总表" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="迷宫导航_全实验总表" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="加法探针_全实验总表" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="迷宫导航_全实验总表" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>